<commit_message>
abandoned carts: weekly 2026-10-03
</commit_message>
<xml_diff>
--- a/reports/abandoned-carts/abandoned_carts_weekly_2026-09-21_2026-09-27.xlsx
+++ b/reports/abandoned-carts/abandoned_carts_weekly_2026-09-21_2026-09-27.xlsx
@@ -1043,7 +1043,7 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>How this was built (Shopify Admin API, pulled 03 Oct 2026 14:26 IST; blue = pulled values, black = formulas):</t>
+          <t>How this was built (Shopify Admin API, pulled 03 Oct 2026 15:39 IST; blue = pulled values, black = formulas):</t>
         </is>
       </c>
     </row>
@@ -1722,10 +1722,10 @@
         <v>0</v>
       </c>
       <c r="T10" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U10" s="6" t="n">
-        <v>191394</v>
+        <v>165384</v>
       </c>
     </row>
     <row r="11">

</xml_diff>